<commit_message>
Auto backup 2026-07-01 09:35:02
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Sales Reports 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78846104-3D74-4972-B123-94272BFE4BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D93170D-8994-426E-8834-C90E9E6D7D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5190" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5183" uniqueCount="594">
   <si>
     <t>Sale-wise Profit Report</t>
   </si>
@@ -1820,6 +1820,15 @@
   </si>
   <si>
     <t>Local Charges in june 9821/3 = 3273.66</t>
+  </si>
+  <si>
+    <t>INV 00091993 2633.78 NZ$ @2.15 CTF Newzealand</t>
+  </si>
+  <si>
+    <t>Collection and delivery Commision Abdul Khan</t>
+  </si>
+  <si>
+    <t>Dubai Office Exp in june 14952.5/3 = 4984.16</t>
   </si>
 </sst>
 </file>
@@ -1969,7 +1978,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2047,6 +2056,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2062,377 +2072,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{7AF396E0-14CD-4B92-AB27-039AE1E776EB}"/>
   </cellStyles>
-  <dxfs count="90">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="53">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -22176,7 +21816,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A6BDDCE-7628-4239-A22E-AFC54CBF13AA}">
-  <dimension ref="A1:L232"/>
+  <dimension ref="A1:L230"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -27386,19 +27026,19 @@
         <v>3069.44</v>
       </c>
       <c r="G131" s="13">
-        <f t="shared" ref="G131:G194" si="4">F131/11</f>
+        <f t="shared" ref="G131:G191" si="4">F131/11</f>
         <v>279.04000000000002</v>
       </c>
       <c r="H131" s="13">
-        <f t="shared" ref="H131:H194" si="5">F131-G131</f>
+        <f t="shared" ref="H131:H191" si="5">F131-G131</f>
         <v>2790.4</v>
       </c>
       <c r="I131" s="13">
-        <f t="shared" ref="I131:I194" si="6">E131-H131</f>
+        <f t="shared" ref="I131:I191" si="6">E131-H131</f>
         <v>1234.5999999999999</v>
       </c>
       <c r="J131" s="14">
-        <f t="shared" ref="J131:J194" si="7">(E131-H131)/H131</f>
+        <f t="shared" ref="J131:J191" si="7">(E131-H131)/H131</f>
         <v>0.44244552752293576</v>
       </c>
       <c r="K131" s="10" t="s">
@@ -29768,38 +29408,38 @@
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B191" s="10" t="s">
-        <v>15</v>
+        <v>552</v>
       </c>
       <c r="C191" s="23" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="D191" s="10" t="s">
-        <v>547</v>
+        <v>17</v>
       </c>
       <c r="E191" s="10">
-        <v>1400</v>
+        <v>11600</v>
       </c>
       <c r="F191" s="10">
-        <v>1108.27</v>
+        <v>10527.57</v>
       </c>
       <c r="G191" s="13">
         <f t="shared" si="4"/>
-        <v>100.75181818181818</v>
+        <v>957.05181818181813</v>
       </c>
       <c r="H191" s="13">
         <f t="shared" si="5"/>
-        <v>1007.5181818181818</v>
+        <v>9570.5181818181809</v>
       </c>
       <c r="I191" s="13">
         <f t="shared" si="6"/>
-        <v>392.4818181818182</v>
+        <v>2029.4818181818191</v>
       </c>
       <c r="J191" s="14">
         <f t="shared" si="7"/>
-        <v>0.38955308724408316</v>
+        <v>0.21205558357721691</v>
       </c>
       <c r="K191" s="10" t="s">
         <v>18</v>
@@ -29808,38 +29448,38 @@
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B192" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C192" s="23" t="s">
-        <v>548</v>
+        <v>276</v>
+      </c>
+      <c r="C192" s="23">
+        <v>39784450551</v>
       </c>
       <c r="D192" s="10" t="s">
-        <v>547</v>
+        <v>17</v>
       </c>
       <c r="E192" s="10">
-        <v>1400</v>
+        <v>4175</v>
       </c>
       <c r="F192" s="10">
-        <v>932.94</v>
+        <v>3143.18</v>
       </c>
       <c r="G192" s="13">
-        <f t="shared" si="4"/>
-        <v>84.812727272727273</v>
+        <f>F192/11</f>
+        <v>285.74363636363637</v>
       </c>
       <c r="H192" s="13">
-        <f t="shared" si="5"/>
-        <v>848.12727272727284</v>
+        <f>F192-G192</f>
+        <v>2857.4363636363632</v>
       </c>
       <c r="I192" s="13">
-        <f t="shared" si="6"/>
-        <v>551.87272727272716</v>
+        <f>E192-H192</f>
+        <v>1317.5636363636368</v>
       </c>
       <c r="J192" s="14">
-        <f t="shared" si="7"/>
-        <v>0.65069565030977317</v>
+        <f>(E192-H192)/H192</f>
+        <v>0.4610999051915578</v>
       </c>
       <c r="K192" s="10" t="s">
         <v>18</v>
@@ -29848,38 +29488,38 @@
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="B193" s="10" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="C193" s="23" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="D193" s="10" t="s">
-        <v>547</v>
+        <v>561</v>
       </c>
       <c r="E193" s="10">
-        <v>1400</v>
+        <v>2070</v>
       </c>
       <c r="F193" s="10">
-        <v>1108.27</v>
+        <v>1527.53</v>
       </c>
       <c r="G193" s="13">
-        <f t="shared" si="4"/>
-        <v>100.75181818181818</v>
+        <f>F193/11</f>
+        <v>138.86636363636364</v>
       </c>
       <c r="H193" s="13">
-        <f t="shared" si="5"/>
-        <v>1007.5181818181818</v>
+        <f>F193-G193</f>
+        <v>1388.6636363636362</v>
       </c>
       <c r="I193" s="13">
-        <f t="shared" si="6"/>
-        <v>392.4818181818182</v>
+        <f>E193-H193</f>
+        <v>681.33636363636379</v>
       </c>
       <c r="J193" s="14">
-        <f t="shared" si="7"/>
-        <v>0.38955308724408316</v>
+        <f>(E193-H193)/H193</f>
+        <v>0.49064175499008217</v>
       </c>
       <c r="K193" s="10" t="s">
         <v>18</v>
@@ -29891,35 +29531,35 @@
         <v>46202</v>
       </c>
       <c r="B194" s="10" t="s">
-        <v>552</v>
+        <v>145</v>
       </c>
       <c r="C194" s="23" t="s">
-        <v>553</v>
+        <v>562</v>
       </c>
       <c r="D194" s="10" t="s">
-        <v>17</v>
+        <v>561</v>
       </c>
       <c r="E194" s="10">
-        <v>11600</v>
+        <v>2070</v>
       </c>
       <c r="F194" s="10">
-        <v>10527.57</v>
+        <v>1527.53</v>
       </c>
       <c r="G194" s="13">
-        <f t="shared" si="4"/>
-        <v>957.05181818181813</v>
+        <f>F194/11</f>
+        <v>138.86636363636364</v>
       </c>
       <c r="H194" s="13">
-        <f t="shared" si="5"/>
-        <v>9570.5181818181809</v>
+        <f>F194-G194</f>
+        <v>1388.6636363636362</v>
       </c>
       <c r="I194" s="13">
-        <f t="shared" si="6"/>
-        <v>2029.4818181818191</v>
+        <f>E194-H194</f>
+        <v>681.33636363636379</v>
       </c>
       <c r="J194" s="14">
-        <f t="shared" si="7"/>
-        <v>0.21205558357721691</v>
+        <f>(E194-H194)/H194</f>
+        <v>0.49064175499008217</v>
       </c>
       <c r="K194" s="10" t="s">
         <v>18</v>
@@ -29928,38 +29568,38 @@
     </row>
     <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="B195" s="10" t="s">
         <v>276</v>
       </c>
       <c r="C195" s="23">
-        <v>39784450551</v>
+        <v>19670053861</v>
       </c>
       <c r="D195" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E195" s="10">
-        <v>4175</v>
+        <v>4000</v>
       </c>
       <c r="F195" s="10">
-        <v>3143.18</v>
+        <v>3115</v>
       </c>
       <c r="G195" s="13">
         <f>F195/11</f>
-        <v>285.74363636363637</v>
+        <v>283.18181818181819</v>
       </c>
       <c r="H195" s="13">
         <f>F195-G195</f>
-        <v>2857.4363636363632</v>
+        <v>2831.818181818182</v>
       </c>
       <c r="I195" s="13">
         <f>E195-H195</f>
-        <v>1317.5636363636368</v>
+        <v>1168.181818181818</v>
       </c>
       <c r="J195" s="14">
         <f>(E195-H195)/H195</f>
-        <v>0.4610999051915578</v>
+        <v>0.41252006420545739</v>
       </c>
       <c r="K195" s="10" t="s">
         <v>18</v>
@@ -29968,38 +29608,38 @@
     </row>
     <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="B196" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="C196" s="23" t="s">
-        <v>560</v>
+        <v>276</v>
+      </c>
+      <c r="C196" s="23">
+        <v>29151959754</v>
       </c>
       <c r="D196" s="10" t="s">
-        <v>561</v>
+        <v>17</v>
       </c>
       <c r="E196" s="10">
-        <v>2070</v>
+        <v>4000</v>
       </c>
       <c r="F196" s="10">
-        <v>1527.53</v>
+        <v>3115</v>
       </c>
       <c r="G196" s="13">
         <f>F196/11</f>
-        <v>138.86636363636364</v>
+        <v>283.18181818181819</v>
       </c>
       <c r="H196" s="13">
         <f>F196-G196</f>
-        <v>1388.6636363636362</v>
+        <v>2831.818181818182</v>
       </c>
       <c r="I196" s="13">
         <f>E196-H196</f>
-        <v>681.33636363636379</v>
+        <v>1168.181818181818</v>
       </c>
       <c r="J196" s="14">
         <f>(E196-H196)/H196</f>
-        <v>0.49064175499008217</v>
+        <v>0.41252006420545739</v>
       </c>
       <c r="K196" s="10" t="s">
         <v>18</v>
@@ -30008,38 +29648,38 @@
     </row>
     <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="B197" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="C197" s="23" t="s">
-        <v>562</v>
+        <v>276</v>
+      </c>
+      <c r="C197" s="23">
+        <v>29690452568</v>
       </c>
       <c r="D197" s="10" t="s">
-        <v>561</v>
+        <v>17</v>
       </c>
       <c r="E197" s="10">
-        <v>2070</v>
+        <v>4000</v>
       </c>
       <c r="F197" s="10">
-        <v>1527.53</v>
+        <v>3115</v>
       </c>
       <c r="G197" s="13">
         <f>F197/11</f>
-        <v>138.86636363636364</v>
+        <v>283.18181818181819</v>
       </c>
       <c r="H197" s="13">
         <f>F197-G197</f>
-        <v>1388.6636363636362</v>
+        <v>2831.818181818182</v>
       </c>
       <c r="I197" s="13">
         <f>E197-H197</f>
-        <v>681.33636363636379</v>
+        <v>1168.181818181818</v>
       </c>
       <c r="J197" s="14">
         <f>(E197-H197)/H197</f>
-        <v>0.49064175499008217</v>
+        <v>0.41252006420545739</v>
       </c>
       <c r="K197" s="10" t="s">
         <v>18</v>
@@ -30054,7 +29694,7 @@
         <v>276</v>
       </c>
       <c r="C198" s="23">
-        <v>19670053861</v>
+        <v>41511018445</v>
       </c>
       <c r="D198" s="10" t="s">
         <v>17</v>
@@ -30094,7 +29734,7 @@
         <v>276</v>
       </c>
       <c r="C199" s="23">
-        <v>29151959754</v>
+        <v>41539033418</v>
       </c>
       <c r="D199" s="10" t="s">
         <v>17</v>
@@ -30134,7 +29774,7 @@
         <v>276</v>
       </c>
       <c r="C200" s="23">
-        <v>29690452568</v>
+        <v>41614067465</v>
       </c>
       <c r="D200" s="10" t="s">
         <v>17</v>
@@ -30174,7 +29814,7 @@
         <v>276</v>
       </c>
       <c r="C201" s="23">
-        <v>41511018445</v>
+        <v>41745009481</v>
       </c>
       <c r="D201" s="10" t="s">
         <v>17</v>
@@ -30214,7 +29854,7 @@
         <v>276</v>
       </c>
       <c r="C202" s="23">
-        <v>41539033418</v>
+        <v>51559056134</v>
       </c>
       <c r="D202" s="10" t="s">
         <v>17</v>
@@ -30254,7 +29894,7 @@
         <v>276</v>
       </c>
       <c r="C203" s="23">
-        <v>41614067465</v>
+        <v>61670053428</v>
       </c>
       <c r="D203" s="10" t="s">
         <v>17</v>
@@ -30294,7 +29934,7 @@
         <v>276</v>
       </c>
       <c r="C204" s="23">
-        <v>41745009481</v>
+        <v>61699071496</v>
       </c>
       <c r="D204" s="10" t="s">
         <v>17</v>
@@ -30334,7 +29974,7 @@
         <v>276</v>
       </c>
       <c r="C205" s="23">
-        <v>51559056134</v>
+        <v>69548862359</v>
       </c>
       <c r="D205" s="10" t="s">
         <v>17</v>
@@ -30374,7 +30014,7 @@
         <v>276</v>
       </c>
       <c r="C206" s="23">
-        <v>61670053428</v>
+        <v>79645154464</v>
       </c>
       <c r="D206" s="10" t="s">
         <v>17</v>
@@ -30414,7 +30054,7 @@
         <v>276</v>
       </c>
       <c r="C207" s="23">
-        <v>61699071496</v>
+        <v>89048444551</v>
       </c>
       <c r="D207" s="10" t="s">
         <v>17</v>
@@ -30447,320 +30087,208 @@
       <c r="L207" s="10"/>
     </row>
     <row r="208" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A208" s="15">
-        <v>46203</v>
-      </c>
-      <c r="B208" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="C208" s="23">
-        <v>69548862359</v>
-      </c>
-      <c r="D208" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E208" s="10">
-        <v>4000</v>
-      </c>
-      <c r="F208" s="10">
-        <v>3115</v>
-      </c>
-      <c r="G208" s="13">
-        <f>F208/11</f>
-        <v>283.18181818181819</v>
-      </c>
-      <c r="H208" s="13">
-        <f>F208-G208</f>
-        <v>2831.818181818182</v>
-      </c>
-      <c r="I208" s="13">
-        <f>E208-H208</f>
-        <v>1168.181818181818</v>
-      </c>
-      <c r="J208" s="14">
-        <f>(E208-H208)/H208</f>
-        <v>0.41252006420545739</v>
-      </c>
-      <c r="K208" s="10" t="s">
-        <v>18</v>
-      </c>
+      <c r="E208" s="11" t="s">
+        <v>567</v>
+      </c>
+      <c r="F208" s="11" t="s">
+        <v>568</v>
+      </c>
+      <c r="G208" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="H208" s="12" t="s">
+        <v>570</v>
+      </c>
+      <c r="I208" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="J208" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="K208" s="10"/>
       <c r="L208" s="10"/>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A209" s="15">
-        <v>46203</v>
-      </c>
-      <c r="B209" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="C209" s="23">
-        <v>79645154464</v>
-      </c>
-      <c r="D209" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E209" s="10">
-        <v>4000</v>
-      </c>
-      <c r="F209" s="10">
-        <v>3115</v>
-      </c>
-      <c r="G209" s="13">
-        <f>F209/11</f>
-        <v>283.18181818181819</v>
-      </c>
-      <c r="H209" s="13">
-        <f>F209-G209</f>
-        <v>2831.818181818182</v>
-      </c>
-      <c r="I209" s="13">
-        <f>E209-H209</f>
-        <v>1168.181818181818</v>
-      </c>
-      <c r="J209" s="14">
-        <f>(E209-H209)/H209</f>
-        <v>0.41252006420545739</v>
-      </c>
-      <c r="K209" s="10" t="s">
-        <v>18</v>
-      </c>
+    <row r="209" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E209" s="7">
+        <f>SUM(E2:E208)</f>
+        <v>653134.99</v>
+      </c>
+      <c r="F209" s="7">
+        <f>SUM(F2:F208)</f>
+        <v>557419.34</v>
+      </c>
+      <c r="G209" s="8">
+        <f>SUM(G2:G208)</f>
+        <v>50674.485454545407</v>
+      </c>
+      <c r="H209" s="8">
+        <f>SUM(H2:H208)</f>
+        <v>506744.85454545484</v>
+      </c>
+      <c r="I209" s="8">
+        <f>SUM(I2:I208)</f>
+        <v>146390.13545454555</v>
+      </c>
+      <c r="J209" s="9">
+        <f>AVERAGE(J2:J208)</f>
+        <v>0.34090331528920426</v>
+      </c>
+      <c r="K209" s="10"/>
       <c r="L209" s="10"/>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A210" s="15">
-        <v>46203</v>
-      </c>
-      <c r="B210" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="C210" s="23">
-        <v>89048444551</v>
-      </c>
-      <c r="D210" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E210" s="10">
-        <v>4000</v>
-      </c>
-      <c r="F210" s="10">
-        <v>3115</v>
-      </c>
-      <c r="G210" s="13">
-        <f>F210/11</f>
-        <v>283.18181818181819</v>
-      </c>
-      <c r="H210" s="13">
-        <f>F210-G210</f>
-        <v>2831.818181818182</v>
-      </c>
-      <c r="I210" s="13">
-        <f>E210-H210</f>
-        <v>1168.181818181818</v>
-      </c>
-      <c r="J210" s="14">
-        <f>(E210-H210)/H210</f>
-        <v>0.41252006420545739</v>
-      </c>
-      <c r="K210" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="L210" s="10"/>
-    </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="E211" s="11" t="s">
-        <v>567</v>
-      </c>
-      <c r="F211" s="11" t="s">
-        <v>568</v>
-      </c>
-      <c r="G211" s="12" t="s">
-        <v>569</v>
-      </c>
-      <c r="H211" s="12" t="s">
-        <v>570</v>
-      </c>
-      <c r="I211" s="12" t="s">
-        <v>571</v>
-      </c>
-      <c r="J211" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="K211" s="10"/>
-      <c r="L211" s="10"/>
-    </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="E212" s="7">
-        <f>SUM(E2:E211)</f>
-        <v>657334.99</v>
-      </c>
-      <c r="F212" s="7">
-        <f>SUM(F2:F211)</f>
-        <v>560568.82000000007</v>
-      </c>
-      <c r="G212" s="8">
-        <f>SUM(G2:G211)</f>
-        <v>50960.801818181768</v>
-      </c>
-      <c r="H212" s="8">
-        <f>SUM(H2:H211)</f>
-        <v>509608.01818181848</v>
-      </c>
-      <c r="I212" s="8">
-        <f>SUM(I2:I211)</f>
-        <v>147726.97181818192</v>
-      </c>
-      <c r="J212" s="9">
-        <f>AVERAGE(J2:J211)</f>
-        <v>0.34285112332236367</v>
-      </c>
-      <c r="K212" s="10"/>
-      <c r="L212" s="10"/>
-    </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B216" s="41" t="s">
+    <row r="213" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B213" s="42" t="s">
         <v>583</v>
       </c>
+      <c r="C213" s="21">
+        <v>10691.07</v>
+      </c>
+    </row>
+    <row r="214" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B214" s="43" t="s">
+        <v>584</v>
+      </c>
+      <c r="C214" s="21">
+        <v>15682.45</v>
+      </c>
+    </row>
+    <row r="215" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B215" s="43" t="s">
+        <v>585</v>
+      </c>
+      <c r="C215" s="21">
+        <v>11863.87</v>
+      </c>
+    </row>
+    <row r="216" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B216" s="43" t="s">
+        <v>590</v>
+      </c>
       <c r="C216" s="21">
-        <v>10691.07</v>
-      </c>
-    </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B217" s="42" t="s">
-        <v>584</v>
+        <v>3273.66</v>
+      </c>
+    </row>
+    <row r="217" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B217" s="43" t="s">
+        <v>586</v>
       </c>
       <c r="C217" s="21">
-        <v>15682.45</v>
-      </c>
-    </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B218" s="42" t="s">
-        <v>585</v>
+        <v>15154.99</v>
+      </c>
+    </row>
+    <row r="218" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B218" s="43" t="s">
+        <v>576</v>
       </c>
       <c r="C218" s="21">
-        <v>11863.87</v>
-      </c>
-    </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B219" s="42" t="s">
-        <v>590</v>
-      </c>
-      <c r="C219" s="21">
-        <v>3273.66</v>
-      </c>
-    </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B220" s="42" t="s">
-        <v>586</v>
+        <v>10140</v>
+      </c>
+    </row>
+    <row r="219" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B219" s="43" t="s">
+        <v>587</v>
+      </c>
+      <c r="C219" s="32">
+        <v>12303.19</v>
+      </c>
+    </row>
+    <row r="220" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B220" s="43" t="s">
+        <v>577</v>
       </c>
       <c r="C220" s="21">
-        <v>15154.99</v>
-      </c>
-    </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B221" s="42" t="s">
-        <v>576</v>
+        <v>6337.5</v>
+      </c>
+    </row>
+    <row r="221" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B221" s="43" t="s">
+        <v>578</v>
       </c>
       <c r="C221" s="21">
-        <v>10140</v>
-      </c>
-    </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B222" s="42" t="s">
-        <v>587</v>
-      </c>
-      <c r="C222" s="32">
-        <v>12303.19</v>
-      </c>
-    </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B223" s="42" t="s">
-        <v>577</v>
+        <v>3727.36</v>
+      </c>
+    </row>
+    <row r="222" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B222" s="43" t="s">
+        <v>579</v>
+      </c>
+      <c r="C222" s="21">
+        <v>3727.37</v>
+      </c>
+    </row>
+    <row r="223" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B223" s="43" t="s">
+        <v>580</v>
       </c>
       <c r="C223" s="21">
-        <v>6337.5</v>
-      </c>
-    </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B224" s="42" t="s">
-        <v>578</v>
+        <v>1013.5</v>
+      </c>
+    </row>
+    <row r="224" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B224" s="43" t="s">
+        <v>581</v>
       </c>
       <c r="C224" s="21">
-        <v>3727.36</v>
+        <v>320</v>
       </c>
     </row>
     <row r="225" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B225" s="42" t="s">
-        <v>579</v>
+      <c r="B225" s="43" t="s">
+        <v>582</v>
       </c>
       <c r="C225" s="21">
-        <v>3727.37</v>
+        <v>256</v>
       </c>
     </row>
     <row r="226" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B226" s="42" t="s">
-        <v>580</v>
+      <c r="B226" s="10" t="s">
+        <v>593</v>
       </c>
       <c r="C226" s="21">
-        <v>1013.5</v>
+        <v>4984.16</v>
       </c>
     </row>
     <row r="227" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B227" s="42" t="s">
-        <v>581</v>
-      </c>
-      <c r="C227" s="21">
-        <v>320</v>
-      </c>
+      <c r="B227" s="10"/>
+      <c r="C227" s="21"/>
     </row>
     <row r="228" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B228" s="42" t="s">
-        <v>582</v>
-      </c>
-      <c r="C228" s="21">
-        <v>256</v>
+      <c r="B228" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="C228" s="5">
+        <f>SUM(C213:C227)</f>
+        <v>99475.12000000001</v>
       </c>
     </row>
     <row r="229" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B229" s="10"/>
       <c r="C229" s="21"/>
     </row>
-    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B230" s="5" t="s">
-        <v>588</v>
-      </c>
-      <c r="C230" s="5">
-        <f>SUM(C216:C229)</f>
-        <v>94490.96</v>
-      </c>
-    </row>
-    <row r="231" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B231" s="10"/>
-      <c r="C231" s="21"/>
-    </row>
-    <row r="232" spans="2:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="B232" s="43" t="s">
+    <row r="230" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B230" s="44" t="s">
         <v>589</v>
       </c>
-      <c r="C232" s="44">
-        <f>I212-C230</f>
-        <v>53236.011818181913</v>
+      <c r="C230" s="45">
+        <f>I209-C228</f>
+        <v>46915.015454545544</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C222">
+  <conditionalFormatting sqref="C219">
     <cfRule type="duplicateValues" dxfId="47" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C222">
+  <conditionalFormatting sqref="C219">
     <cfRule type="duplicateValues" dxfId="46" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C231 C1:C229 C233:C1048576">
+  <conditionalFormatting sqref="C229 C1:C227 C231:C1048576">
     <cfRule type="duplicateValues" dxfId="45" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C210">
-    <cfRule type="duplicateValues" dxfId="44" priority="39"/>
+  <conditionalFormatting sqref="C218:C222">
+    <cfRule type="duplicateValues" dxfId="44" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C221:C225">
-    <cfRule type="duplicateValues" dxfId="43" priority="1"/>
+  <conditionalFormatting sqref="C2:C207">
+    <cfRule type="duplicateValues" dxfId="0" priority="43"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30768,11 +30296,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B5EA52-4A09-4771-8155-97F59FDF1D1A}">
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="22" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" customWidth="1"/>
     <col min="3" max="3" width="35" style="22" customWidth="1"/>
     <col min="4" max="4" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.5703125" customWidth="1"/>
@@ -34144,13 +33672,40 @@
       <c r="K87" s="10"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B94" s="42" t="s">
+      <c r="B94" s="43" t="s">
         <v>590</v>
+      </c>
+      <c r="C94" s="22">
+        <v>3273.66</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B95" s="41" t="s">
+        <v>591</v>
+      </c>
+      <c r="C95" s="22">
+        <v>5662.62</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B96" s="41" t="s">
+        <v>592</v>
+      </c>
+      <c r="C96" s="22">
+        <v>5613.5</v>
+      </c>
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>593</v>
+      </c>
+      <c r="C97" s="22">
+        <v>4984.16</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C85">
-    <cfRule type="duplicateValues" dxfId="42" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -35910,12 +35465,15 @@
       <c r="C60" s="33"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="42" t="s">
+      <c r="B61" s="43" t="s">
         <v>590</v>
       </c>
       <c r="C61" s="33"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>593</v>
+      </c>
       <c r="C62" s="33"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
@@ -36073,13 +35631,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C53">
-    <cfRule type="duplicateValues" dxfId="41" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C60:C113">
-    <cfRule type="duplicateValues" dxfId="40" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="39" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -44453,7 +44011,7 @@
       <c r="J262" s="10"/>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B268" s="42" t="s">
+      <c r="B268" s="43" t="s">
         <v>590</v>
       </c>
     </row>
@@ -44678,10 +44236,10 @@
     <sortCondition ref="I2:I260"/>
   </sortState>
   <conditionalFormatting sqref="C2:C260">
-    <cfRule type="duplicateValues" dxfId="38" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="37" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -46342,115 +45900,115 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C3">
-    <cfRule type="duplicateValues" dxfId="36" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C5">
-    <cfRule type="duplicateValues" dxfId="35" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C5">
-    <cfRule type="duplicateValues" dxfId="34" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C9">
-    <cfRule type="duplicateValues" dxfId="33" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C9">
-    <cfRule type="duplicateValues" dxfId="32" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="30" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:C15">
-    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:C15">
-    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:C17">
-    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:C17">
-    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="20" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C21">
-    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C21">
-    <cfRule type="duplicateValues" dxfId="18" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:C27">
-    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:C27">
-    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C33">
-    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C33">
-    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35:C38">
-    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35:C38">
-    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C39:C42">
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C39:C42">
-    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C44">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C44">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C50:C103">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C44 C46:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 10:05:02
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Sales Reports 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D93170D-8994-426E-8834-C90E9E6D7D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F283EFE7-8798-47E2-9B73-044008C87A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5183" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5186" uniqueCount="595">
   <si>
     <t>Sale-wise Profit Report</t>
   </si>
@@ -1829,6 +1829,9 @@
   </si>
   <si>
     <t>Dubai Office Exp in june 14952.5/3 = 4984.16</t>
+  </si>
+  <si>
+    <t>Dxb &amp; Khi Salary Exp in june  21135.44/3 = 7045.14</t>
   </si>
 </sst>
 </file>
@@ -1978,7 +1981,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2061,6 +2064,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -21816,7 +21820,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A6BDDCE-7628-4239-A22E-AFC54CBF13AA}">
-  <dimension ref="A1:L230"/>
+  <dimension ref="A1:L231"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -30177,118 +30181,126 @@
       </c>
     </row>
     <row r="218" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B218" s="43" t="s">
-        <v>576</v>
+      <c r="B218" s="44" t="s">
+        <v>594</v>
       </c>
       <c r="C218" s="21">
-        <v>10140</v>
+        <v>7045.14</v>
       </c>
     </row>
     <row r="219" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B219" s="43" t="s">
-        <v>587</v>
-      </c>
-      <c r="C219" s="32">
-        <v>12303.19</v>
+        <v>576</v>
+      </c>
+      <c r="C219" s="21">
+        <v>10140</v>
       </c>
     </row>
     <row r="220" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B220" s="43" t="s">
-        <v>577</v>
-      </c>
-      <c r="C220" s="21">
-        <v>6337.5</v>
+        <v>587</v>
+      </c>
+      <c r="C220" s="32">
+        <v>12303.19</v>
       </c>
     </row>
     <row r="221" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B221" s="43" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C221" s="21">
-        <v>3727.36</v>
+        <v>6337.5</v>
       </c>
     </row>
     <row r="222" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B222" s="43" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C222" s="21">
-        <v>3727.37</v>
+        <v>3727.36</v>
       </c>
     </row>
     <row r="223" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B223" s="43" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C223" s="21">
-        <v>1013.5</v>
+        <v>3727.37</v>
       </c>
     </row>
     <row r="224" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B224" s="43" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C224" s="21">
-        <v>320</v>
+        <v>1013.5</v>
       </c>
     </row>
     <row r="225" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B225" s="43" t="s">
+        <v>581</v>
+      </c>
+      <c r="C225" s="21">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B226" s="43" t="s">
         <v>582</v>
       </c>
-      <c r="C225" s="21">
+      <c r="C226" s="21">
         <v>256</v>
       </c>
     </row>
-    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B226" s="10" t="s">
+    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B227" s="10" t="s">
         <v>593</v>
       </c>
-      <c r="C226" s="21">
+      <c r="C227" s="21">
         <v>4984.16</v>
       </c>
     </row>
-    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B227" s="10"/>
-      <c r="C227" s="21"/>
-    </row>
     <row r="228" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B228" s="5" t="s">
+      <c r="B228" s="10"/>
+      <c r="C228" s="21"/>
+    </row>
+    <row r="229" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B229" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="C228" s="5">
-        <f>SUM(C213:C227)</f>
-        <v>99475.12000000001</v>
-      </c>
-    </row>
-    <row r="229" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B229" s="10"/>
-      <c r="C229" s="21"/>
-    </row>
-    <row r="230" spans="2:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="B230" s="44" t="s">
+      <c r="C229" s="5">
+        <f>SUM(C213:C228)</f>
+        <v>106520.26</v>
+      </c>
+    </row>
+    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B230" s="10"/>
+      <c r="C230" s="21"/>
+    </row>
+    <row r="231" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B231" s="45" t="s">
         <v>589</v>
       </c>
-      <c r="C230" s="45">
-        <f>I209-C228</f>
-        <v>46915.015454545544</v>
+      <c r="C231" s="46">
+        <f>I209-C229</f>
+        <v>39869.875454545559</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C219">
+  <conditionalFormatting sqref="C220">
     <cfRule type="duplicateValues" dxfId="47" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C219">
+  <conditionalFormatting sqref="C220">
     <cfRule type="duplicateValues" dxfId="46" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C229 C1:C227 C231:C1048576">
+  <conditionalFormatting sqref="C230 C1:C228 C232:C1048576">
     <cfRule type="duplicateValues" dxfId="45" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C218:C222">
+  <conditionalFormatting sqref="C219:C223">
     <cfRule type="duplicateValues" dxfId="44" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C207">
-    <cfRule type="duplicateValues" dxfId="0" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="43"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30296,7 +30308,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B5EA52-4A09-4771-8155-97F59FDF1D1A}">
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="22" customWidth="1"/>
@@ -33703,9 +33715,17 @@
         <v>4984.16</v>
       </c>
     </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B98" s="44" t="s">
+        <v>594</v>
+      </c>
+      <c r="C98" s="22">
+        <v>7045.14</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C85">
-    <cfRule type="duplicateValues" dxfId="43" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -33717,7 +33737,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="22" customWidth="1"/>
-    <col min="2" max="2" width="41" customWidth="1"/>
+    <col min="2" max="2" width="44.7109375" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" style="22" customWidth="1"/>
     <col min="4" max="4" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" customWidth="1"/>
@@ -35477,6 +35497,9 @@
       <c r="C62" s="33"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B63" s="44" t="s">
+        <v>594</v>
+      </c>
       <c r="C63" s="34"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -35631,13 +35654,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C53">
-    <cfRule type="duplicateValues" dxfId="42" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C60:C113">
-    <cfRule type="duplicateValues" dxfId="41" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -44236,10 +44259,10 @@
     <sortCondition ref="I2:I260"/>
   </sortState>
   <conditionalFormatting sqref="C2:C260">
-    <cfRule type="duplicateValues" dxfId="39" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="38" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -45900,115 +45923,115 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C3">
-    <cfRule type="duplicateValues" dxfId="37" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C5">
-    <cfRule type="duplicateValues" dxfId="36" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C5">
-    <cfRule type="duplicateValues" dxfId="35" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C9">
-    <cfRule type="duplicateValues" dxfId="34" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C9">
-    <cfRule type="duplicateValues" dxfId="33" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="32" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="31" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="30" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="29" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:C15">
-    <cfRule type="duplicateValues" dxfId="28" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:C15">
-    <cfRule type="duplicateValues" dxfId="27" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:C17">
-    <cfRule type="duplicateValues" dxfId="26" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:C17">
-    <cfRule type="duplicateValues" dxfId="25" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="24" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="23" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="22" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="21" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C21">
-    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C21">
-    <cfRule type="duplicateValues" dxfId="19" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:C27">
-    <cfRule type="duplicateValues" dxfId="18" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:C27">
-    <cfRule type="duplicateValues" dxfId="17" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C33">
-    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C33">
-    <cfRule type="duplicateValues" dxfId="15" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="14" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="13" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35:C38">
-    <cfRule type="duplicateValues" dxfId="12" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35:C38">
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C39:C42">
-    <cfRule type="duplicateValues" dxfId="10" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C39:C42">
-    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C44">
-    <cfRule type="duplicateValues" dxfId="6" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C44">
-    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C50:C103">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C44 C46:C1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 10:35:02
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Sales Reports 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F283EFE7-8798-47E2-9B73-044008C87A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE7CDBB-3BEF-469B-B34A-9101739440E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5186" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5189" uniqueCount="598">
   <si>
     <t>Sale-wise Profit Report</t>
   </si>
@@ -1832,6 +1832,15 @@
   </si>
   <si>
     <t>Dxb &amp; Khi Salary Exp in june  21135.44/3 = 7045.14</t>
+  </si>
+  <si>
+    <t>Carry Exp</t>
+  </si>
+  <si>
+    <t>408 Shop Exp</t>
+  </si>
+  <si>
+    <t>Karachi Office Exp</t>
   </si>
 </sst>
 </file>
@@ -1981,7 +1990,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2060,6 +2069,9 @@
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -30141,7 +30153,7 @@
       <c r="L209" s="10"/>
     </row>
     <row r="213" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B213" s="42" t="s">
+      <c r="B213" s="43" t="s">
         <v>583</v>
       </c>
       <c r="C213" s="21">
@@ -30149,7 +30161,7 @@
       </c>
     </row>
     <row r="214" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B214" s="43" t="s">
+      <c r="B214" s="44" t="s">
         <v>584</v>
       </c>
       <c r="C214" s="21">
@@ -30157,7 +30169,7 @@
       </c>
     </row>
     <row r="215" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B215" s="43" t="s">
+      <c r="B215" s="44" t="s">
         <v>585</v>
       </c>
       <c r="C215" s="21">
@@ -30165,7 +30177,7 @@
       </c>
     </row>
     <row r="216" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B216" s="43" t="s">
+      <c r="B216" s="44" t="s">
         <v>590</v>
       </c>
       <c r="C216" s="21">
@@ -30173,7 +30185,7 @@
       </c>
     </row>
     <row r="217" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B217" s="43" t="s">
+      <c r="B217" s="44" t="s">
         <v>586</v>
       </c>
       <c r="C217" s="21">
@@ -30181,7 +30193,7 @@
       </c>
     </row>
     <row r="218" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B218" s="44" t="s">
+      <c r="B218" s="45" t="s">
         <v>594</v>
       </c>
       <c r="C218" s="21">
@@ -30189,7 +30201,7 @@
       </c>
     </row>
     <row r="219" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B219" s="43" t="s">
+      <c r="B219" s="44" t="s">
         <v>576</v>
       </c>
       <c r="C219" s="21">
@@ -30197,7 +30209,7 @@
       </c>
     </row>
     <row r="220" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B220" s="43" t="s">
+      <c r="B220" s="44" t="s">
         <v>587</v>
       </c>
       <c r="C220" s="32">
@@ -30205,7 +30217,7 @@
       </c>
     </row>
     <row r="221" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B221" s="43" t="s">
+      <c r="B221" s="44" t="s">
         <v>577</v>
       </c>
       <c r="C221" s="21">
@@ -30213,7 +30225,7 @@
       </c>
     </row>
     <row r="222" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B222" s="43" t="s">
+      <c r="B222" s="44" t="s">
         <v>578</v>
       </c>
       <c r="C222" s="21">
@@ -30221,7 +30233,7 @@
       </c>
     </row>
     <row r="223" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B223" s="43" t="s">
+      <c r="B223" s="44" t="s">
         <v>579</v>
       </c>
       <c r="C223" s="21">
@@ -30229,7 +30241,7 @@
       </c>
     </row>
     <row r="224" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B224" s="43" t="s">
+      <c r="B224" s="44" t="s">
         <v>580</v>
       </c>
       <c r="C224" s="21">
@@ -30237,7 +30249,7 @@
       </c>
     </row>
     <row r="225" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B225" s="43" t="s">
+      <c r="B225" s="44" t="s">
         <v>581</v>
       </c>
       <c r="C225" s="21">
@@ -30245,7 +30257,7 @@
       </c>
     </row>
     <row r="226" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B226" s="43" t="s">
+      <c r="B226" s="44" t="s">
         <v>582</v>
       </c>
       <c r="C226" s="21">
@@ -30278,10 +30290,10 @@
       <c r="C230" s="21"/>
     </row>
     <row r="231" spans="2:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="B231" s="45" t="s">
+      <c r="B231" s="46" t="s">
         <v>589</v>
       </c>
-      <c r="C231" s="46">
+      <c r="C231" s="47">
         <f>I209-C229</f>
         <v>39869.875454545559</v>
       </c>
@@ -33684,7 +33696,7 @@
       <c r="K87" s="10"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B94" s="43" t="s">
+      <c r="B94" s="44" t="s">
         <v>590</v>
       </c>
       <c r="C94" s="22">
@@ -33716,7 +33728,7 @@
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B98" s="44" t="s">
+      <c r="B98" s="45" t="s">
         <v>594</v>
       </c>
       <c r="C98" s="22">
@@ -35485,7 +35497,7 @@
       <c r="C60" s="33"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="43" t="s">
+      <c r="B61" s="44" t="s">
         <v>590</v>
       </c>
       <c r="C61" s="33"/>
@@ -35497,7 +35509,7 @@
       <c r="C62" s="33"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="44" t="s">
+      <c r="B63" s="45" t="s">
         <v>594</v>
       </c>
       <c r="C63" s="34"/>
@@ -44034,7 +44046,7 @@
       <c r="J262" s="10"/>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B268" s="43" t="s">
+      <c r="B268" s="44" t="s">
         <v>590</v>
       </c>
     </row>
@@ -45759,49 +45771,64 @@
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C50" s="33"/>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C51" s="33"/>
     </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C52" s="33"/>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="34"/>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C54" s="33"/>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="33"/>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>595</v>
+      </c>
+      <c r="C53" s="34">
+        <v>8151.89</v>
+      </c>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>596</v>
+      </c>
+      <c r="C54" s="42">
+        <v>1062.01</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>597</v>
+      </c>
+      <c r="C55" s="42">
+        <v>7677</v>
+      </c>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C56" s="33"/>
     </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C57" s="33"/>
     </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C60" s="33"/>
     </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C61" s="33"/>
     </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C62" s="34"/>
     </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C63" s="33"/>
     </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C64" s="33"/>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Auto backup 2026-07-02 03:05:01
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Sales Reports 2025/Sales Report June-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Sales Reports 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219AAD04-B4E6-427C-9FEF-ED731BA8819D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B091008-6629-447F-AAC9-C0A18E7BDA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B6D4EC9A-6888-49F7-BC98-088E7BD35AE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4801" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4826" uniqueCount="608">
   <si>
     <t>Sale-wise Profit Report</t>
   </si>
@@ -1840,7 +1840,37 @@
     <t>408 Shop Exp</t>
   </si>
   <si>
-    <t>Karachi Office Exp</t>
+    <t>Karachi Office Exp 7677/3 =2559</t>
+  </si>
+  <si>
+    <t>ST Usa Business Exp in June-2026</t>
+  </si>
+  <si>
+    <t>21.32 US$ @3.674 Claude AI Charges</t>
+  </si>
+  <si>
+    <t>36.27 US$ @3.674 AWS Charges</t>
+  </si>
+  <si>
+    <t>2-june label 17328 1833.25 US$ @3.674 ST</t>
+  </si>
+  <si>
+    <t>22-june label 17424 &amp; 17511 1833.25 US$ @3.674 ST</t>
+  </si>
+  <si>
+    <t>11-june label 57726 89.69 US$ @3.674 ST</t>
+  </si>
+  <si>
+    <t>Total Profit in ST USA</t>
+  </si>
+  <si>
+    <t>Total Profit in USA</t>
+  </si>
+  <si>
+    <t>Total Profit in Karachi</t>
+  </si>
+  <si>
+    <t>Total Profit in NewZealand</t>
   </si>
 </sst>
 </file>
@@ -1990,7 +2020,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2068,27 +2098,66 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{7AF396E0-14CD-4B92-AB27-039AE1E776EB}"/>
   </cellStyles>
-  <dxfs count="49">
+  <dxfs count="51">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -21784,7 +21853,7 @@
   </sheetData>
   <autoFilter ref="A6:I655" xr:uid="{9BB2F6C6-EF2F-424D-9FFF-ECB06C81F028}"/>
   <conditionalFormatting sqref="C1:C655">
-    <cfRule type="duplicateValues" dxfId="48" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21792,7 +21861,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A6BDDCE-7628-4239-A22E-AFC54CBF13AA}">
-  <dimension ref="A1:L231"/>
+  <dimension ref="A1:L232"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -30113,7 +30182,7 @@
       <c r="L209" s="10"/>
     </row>
     <row r="213" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B213" s="43" t="s">
+      <c r="B213" s="41" t="s">
         <v>583</v>
       </c>
       <c r="C213" s="21">
@@ -30121,7 +30190,7 @@
       </c>
     </row>
     <row r="214" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B214" s="44" t="s">
+      <c r="B214" s="42" t="s">
         <v>584</v>
       </c>
       <c r="C214" s="21">
@@ -30129,7 +30198,7 @@
       </c>
     </row>
     <row r="215" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B215" s="44" t="s">
+      <c r="B215" s="42" t="s">
         <v>585</v>
       </c>
       <c r="C215" s="21">
@@ -30137,7 +30206,7 @@
       </c>
     </row>
     <row r="216" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B216" s="44" t="s">
+      <c r="B216" s="42" t="s">
         <v>590</v>
       </c>
       <c r="C216" s="21">
@@ -30145,132 +30214,142 @@
       </c>
     </row>
     <row r="217" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B217" s="44" t="s">
+      <c r="B217" s="42" t="s">
         <v>586</v>
       </c>
       <c r="C217" s="21">
         <v>15154.99</v>
       </c>
     </row>
-    <row r="218" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B218" s="45" t="s">
+    <row r="218" spans="2:12" s="45" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B218" s="47" t="s">
+        <v>597</v>
+      </c>
+      <c r="C218" s="48">
+        <v>2559</v>
+      </c>
+      <c r="G218" s="3"/>
+      <c r="J218" s="4"/>
+    </row>
+    <row r="219" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B219" s="50" t="s">
         <v>594</v>
       </c>
-      <c r="C218" s="21">
+      <c r="C219" s="21">
         <v>7045.14</v>
       </c>
     </row>
-    <row r="219" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B219" s="44" t="s">
+    <row r="220" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B220" s="42" t="s">
         <v>576</v>
       </c>
-      <c r="C219" s="21">
+      <c r="C220" s="21">
         <v>10140</v>
       </c>
     </row>
-    <row r="220" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B220" s="44" t="s">
+    <row r="221" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B221" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="C220" s="32">
+      <c r="C221" s="32">
         <v>12303.19</v>
       </c>
     </row>
-    <row r="221" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B221" s="44" t="s">
+    <row r="222" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B222" s="42" t="s">
         <v>577</v>
       </c>
-      <c r="C221" s="21">
+      <c r="C222" s="21">
         <v>6337.5</v>
       </c>
     </row>
-    <row r="222" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B222" s="44" t="s">
+    <row r="223" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B223" s="42" t="s">
         <v>578</v>
       </c>
-      <c r="C222" s="21">
+      <c r="C223" s="21">
         <v>3727.36</v>
       </c>
     </row>
-    <row r="223" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B223" s="44" t="s">
+    <row r="224" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B224" s="42" t="s">
         <v>579</v>
       </c>
-      <c r="C223" s="21">
+      <c r="C224" s="21">
         <v>3727.37</v>
       </c>
     </row>
-    <row r="224" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B224" s="44" t="s">
+    <row r="225" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B225" s="42" t="s">
         <v>580</v>
       </c>
-      <c r="C224" s="21">
+      <c r="C225" s="21">
         <v>1013.5</v>
       </c>
     </row>
-    <row r="225" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B225" s="44" t="s">
+    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B226" s="42" t="s">
         <v>581</v>
       </c>
-      <c r="C225" s="21">
+      <c r="C226" s="21">
         <v>320</v>
       </c>
     </row>
-    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B226" s="44" t="s">
+    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B227" s="42" t="s">
         <v>582</v>
       </c>
-      <c r="C226" s="21">
+      <c r="C227" s="21">
         <v>256</v>
       </c>
     </row>
-    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B227" s="10" t="s">
+    <row r="228" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B228" s="10" t="s">
         <v>593</v>
       </c>
-      <c r="C227" s="21">
+      <c r="C228" s="21">
         <v>4984.16</v>
       </c>
     </row>
-    <row r="228" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B228" s="10"/>
-      <c r="C228" s="21"/>
-    </row>
     <row r="229" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B229" s="5" t="s">
+      <c r="B229" s="10"/>
+      <c r="C229" s="21"/>
+    </row>
+    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B230" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="C229" s="5">
-        <f>SUM(C213:C228)</f>
-        <v>106520.26</v>
-      </c>
-    </row>
-    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B230" s="10"/>
-      <c r="C230" s="21"/>
-    </row>
-    <row r="231" spans="2:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="B231" s="46" t="s">
+      <c r="C230" s="5">
+        <f>SUM(C213:C229)</f>
+        <v>109079.26000000001</v>
+      </c>
+    </row>
+    <row r="231" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B231" s="10"/>
+      <c r="C231" s="21"/>
+    </row>
+    <row r="232" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B232" s="43" t="s">
         <v>589</v>
       </c>
-      <c r="C231" s="47">
-        <f>I209-C229</f>
-        <v>39869.875454545559</v>
+      <c r="C232" s="44">
+        <f>I209-C230</f>
+        <v>37310.875454545545</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C207">
-    <cfRule type="duplicateValues" dxfId="47" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="43"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C219:C223">
-    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
+  <conditionalFormatting sqref="C220:C224">
+    <cfRule type="duplicateValues" dxfId="48" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C220">
-    <cfRule type="duplicateValues" dxfId="45" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="4"/>
+  <conditionalFormatting sqref="C221">
+    <cfRule type="duplicateValues" dxfId="47" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C230 C1:C228 C232:C1048576">
-    <cfRule type="duplicateValues" dxfId="43" priority="2"/>
+  <conditionalFormatting sqref="C231 C1:C229 C233:C1048576">
+    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30278,7 +30357,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B5EA52-4A09-4771-8155-97F59FDF1D1A}">
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="22" customWidth="1"/>
@@ -33654,48 +33733,82 @@
       <c r="K87" s="10"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B94" s="44" t="s">
+      <c r="B94" s="42" t="s">
         <v>590</v>
       </c>
-      <c r="C94" s="22">
+      <c r="C94" s="48">
         <v>3273.66</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B95" s="41" t="s">
+      <c r="B95" s="42" t="s">
         <v>591</v>
       </c>
-      <c r="C95" s="22">
+      <c r="C95" s="48">
         <v>5662.62</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B96" s="41" t="s">
+      <c r="B96" s="42" t="s">
         <v>592</v>
       </c>
-      <c r="C96" s="22">
+      <c r="C96" s="48">
         <v>5613.5</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B97" t="s">
+      <c r="B97" s="47" t="s">
         <v>593</v>
       </c>
-      <c r="C97" s="22">
+      <c r="C97" s="48">
         <v>4984.16</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B98" s="45" t="s">
+      <c r="B98" s="50" t="s">
         <v>594</v>
       </c>
-      <c r="C98" s="22">
+      <c r="C98" s="48">
         <v>7045.14</v>
+      </c>
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B99" s="47" t="s">
+        <v>597</v>
+      </c>
+      <c r="C99" s="48">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B100" s="47"/>
+      <c r="C100" s="48"/>
+    </row>
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B101" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="C101" s="5">
+        <f>SUM(C94:C100)</f>
+        <v>29138.079999999998</v>
+      </c>
+    </row>
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B102" s="47"/>
+      <c r="C102" s="48"/>
+    </row>
+    <row r="103" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B103" s="43" t="s">
+        <v>607</v>
+      </c>
+      <c r="C103" s="44">
+        <f>I87-C101</f>
+        <v>107473.27015200008</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C85">
-    <cfRule type="duplicateValues" dxfId="42" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -33707,7 +33820,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="22" customWidth="1"/>
-    <col min="2" max="2" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" style="22" customWidth="1"/>
     <col min="4" max="4" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" customWidth="1"/>
@@ -35455,72 +35568,127 @@
       <c r="C60" s="33"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="44" t="s">
+      <c r="B61" s="51" t="s">
         <v>590</v>
       </c>
-      <c r="C61" s="33"/>
+      <c r="C61" s="54">
+        <v>1636.83</v>
+      </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
+      <c r="B62" s="52" t="s">
         <v>593</v>
       </c>
-      <c r="C62" s="33"/>
+      <c r="C62" s="54">
+        <v>2492.08</v>
+      </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="45" t="s">
+      <c r="B63" s="53" t="s">
         <v>594</v>
       </c>
-      <c r="C63" s="34"/>
+      <c r="C63" s="48">
+        <v>3522.57</v>
+      </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C64" s="33"/>
-    </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="33"/>
-    </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="33"/>
-    </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="33"/>
-    </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="33"/>
-    </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="33"/>
-    </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="33"/>
-    </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="33"/>
-    </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="34"/>
-    </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C73" s="33"/>
-    </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C74" s="33"/>
-    </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="B64" s="42" t="s">
+        <v>601</v>
+      </c>
+      <c r="C64" s="46">
+        <v>3367.68</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B65" s="42" t="s">
+        <v>602</v>
+      </c>
+      <c r="C65" s="46">
+        <v>4542.62</v>
+      </c>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B66" s="42" t="s">
+        <v>603</v>
+      </c>
+      <c r="C66" s="46">
+        <v>164.76</v>
+      </c>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B67" s="52" t="s">
+        <v>597</v>
+      </c>
+      <c r="C67" s="54">
+        <v>1279.5</v>
+      </c>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B68" s="51" t="s">
+        <v>598</v>
+      </c>
+      <c r="C68" s="54">
+        <v>5511</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B69" s="51" t="s">
+        <v>600</v>
+      </c>
+      <c r="C69" s="54">
+        <v>66.62</v>
+      </c>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B70" s="51" t="s">
+        <v>599</v>
+      </c>
+      <c r="C70" s="54">
+        <v>39.159999999999997</v>
+      </c>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="47"/>
+      <c r="C71" s="49"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="C72" s="5">
+        <f>SUM(C61:C71)</f>
+        <v>22622.82</v>
+      </c>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="47"/>
+      <c r="C73" s="49"/>
+    </row>
+    <row r="74" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B74" s="43" t="s">
+        <v>604</v>
+      </c>
+      <c r="C74" s="43">
+        <f>G55-C72</f>
+        <v>2746.2499999999563</v>
+      </c>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C75" s="33"/>
     </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C76" s="33"/>
     </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C77" s="33"/>
     </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C78" s="33"/>
     </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C79" s="34"/>
     </row>
-    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C80" s="33"/>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.25">
@@ -35623,14 +35791,14 @@
       <c r="C113" s="33"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="41" priority="1"/>
+  <conditionalFormatting sqref="C1:C71 C73 C75:C1048576">
+    <cfRule type="duplicateValues" dxfId="43" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C53">
-    <cfRule type="duplicateValues" dxfId="40" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C60:C113">
-    <cfRule type="duplicateValues" dxfId="39" priority="2"/>
+  <conditionalFormatting sqref="C60:C71 C73 C75:C113">
+    <cfRule type="duplicateValues" dxfId="41" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -44004,75 +44172,146 @@
       <c r="J262" s="10"/>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B268" s="44" t="s">
+      <c r="B268" s="51" t="s">
         <v>590</v>
       </c>
+      <c r="C268" s="54">
+        <v>1636.83</v>
+      </c>
+    </row>
+    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B269" s="52" t="s">
+        <v>593</v>
+      </c>
+      <c r="C269" s="54">
+        <v>2492.08</v>
+      </c>
+    </row>
+    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B270" s="53" t="s">
+        <v>594</v>
+      </c>
+      <c r="C270" s="48">
+        <v>3522.57</v>
+      </c>
+    </row>
+    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B271" s="42" t="s">
+        <v>601</v>
+      </c>
+      <c r="C271" s="46">
+        <v>3367.68</v>
+      </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C272" s="33"/>
+      <c r="B272" s="42" t="s">
+        <v>602</v>
+      </c>
+      <c r="C272" s="46">
+        <v>4542.62</v>
+      </c>
       <c r="D272" s="35"/>
     </row>
-    <row r="273" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C273" s="33"/>
+    <row r="273" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B273" s="42" t="s">
+        <v>603</v>
+      </c>
+      <c r="C273" s="46">
+        <v>164.76</v>
+      </c>
       <c r="D273" s="35"/>
     </row>
-    <row r="274" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C274" s="33"/>
+    <row r="274" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B274" s="52" t="s">
+        <v>597</v>
+      </c>
+      <c r="C274" s="54">
+        <v>1279.5</v>
+      </c>
       <c r="D274" s="35"/>
     </row>
-    <row r="275" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C275" s="36"/>
+    <row r="275" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B275" s="51" t="s">
+        <v>598</v>
+      </c>
+      <c r="C275" s="54">
+        <v>5511</v>
+      </c>
       <c r="D275" s="37"/>
     </row>
-    <row r="276" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C276" s="33"/>
+    <row r="276" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B276" s="51" t="s">
+        <v>600</v>
+      </c>
+      <c r="C276" s="54">
+        <v>66.62</v>
+      </c>
       <c r="D276" s="35"/>
     </row>
-    <row r="277" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C277" s="33"/>
+    <row r="277" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B277" s="51" t="s">
+        <v>599</v>
+      </c>
+      <c r="C277" s="54">
+        <v>39.159999999999997</v>
+      </c>
       <c r="D277" s="35"/>
     </row>
-    <row r="278" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C278" s="33"/>
+    <row r="278" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B278" s="47"/>
+      <c r="C278" s="49"/>
       <c r="D278" s="35"/>
     </row>
-    <row r="279" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C279" s="33"/>
+    <row r="279" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B279" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="C279" s="5">
+        <f>SUM(C268:C278)</f>
+        <v>22622.82</v>
+      </c>
       <c r="D279" s="35"/>
     </row>
-    <row r="280" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C280" s="33"/>
+    <row r="280" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B280" s="47"/>
+      <c r="C280" s="49"/>
       <c r="D280" s="35"/>
     </row>
-    <row r="281" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C281" s="33"/>
+    <row r="281" spans="2:4" ht="21" x14ac:dyDescent="0.25">
+      <c r="B281" s="43" t="s">
+        <v>605</v>
+      </c>
+      <c r="C281" s="43">
+        <f>G262-C279</f>
+        <v>26030.559999999925</v>
+      </c>
       <c r="D281" s="35"/>
     </row>
-    <row r="282" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C282" s="33"/>
       <c r="D282" s="35"/>
     </row>
-    <row r="283" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C283" s="33"/>
       <c r="D283" s="35"/>
     </row>
-    <row r="284" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C284" s="36"/>
       <c r="D284" s="37"/>
     </row>
-    <row r="285" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C285" s="33"/>
       <c r="D285" s="35"/>
     </row>
-    <row r="286" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C286" s="33"/>
       <c r="D286" s="35"/>
     </row>
-    <row r="287" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C287" s="33"/>
       <c r="D287" s="35"/>
     </row>
-    <row r="288" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C288" s="33"/>
       <c r="D288" s="35"/>
     </row>
@@ -44228,11 +44467,17 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J260">
     <sortCondition ref="I2:I260"/>
   </sortState>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="38" priority="1"/>
+  <conditionalFormatting sqref="C1:C267 C278 C280 C282:C1048576">
+    <cfRule type="duplicateValues" dxfId="40" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C260">
-    <cfRule type="duplicateValues" dxfId="37" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C268:C277">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C268:C277">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -45739,37 +45984,46 @@
       <c r="C52" s="33"/>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B53" t="s">
+      <c r="B53" s="47" t="s">
         <v>595</v>
       </c>
-      <c r="C53" s="34">
+      <c r="C53" s="48">
         <v>8151.89</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B54" t="s">
+      <c r="B54" s="47" t="s">
         <v>596</v>
       </c>
-      <c r="C54" s="42">
+      <c r="C54" s="32">
         <v>1062.01</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
-        <v>597</v>
-      </c>
-      <c r="C55" s="42">
-        <v>7677</v>
-      </c>
+      <c r="B55" s="47"/>
+      <c r="C55" s="32"/>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C56" s="33"/>
+      <c r="B56" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="C56" s="5">
+        <f>SUM(C53:C55)</f>
+        <v>9213.9</v>
+      </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="33"/>
-    </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C58" s="33"/>
+      <c r="B57" s="47"/>
+      <c r="C57" s="49"/>
+    </row>
+    <row r="58" spans="2:3" ht="21" x14ac:dyDescent="0.25">
+      <c r="B58" s="43" t="s">
+        <v>606</v>
+      </c>
+      <c r="C58" s="44">
+        <f>G47-C56</f>
+        <v>3537.2890909090929</v>
+      </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C59" s="33"/>
@@ -45907,82 +46161,82 @@
       <c r="C103" s="33"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C1:C44 C46:C1048576">
-    <cfRule type="duplicateValues" dxfId="36" priority="3"/>
+  <conditionalFormatting sqref="C1:C44 C46:C55 C57 C59:C1048576">
+    <cfRule type="duplicateValues" dxfId="38" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C3">
-    <cfRule type="duplicateValues" dxfId="35" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C5">
-    <cfRule type="duplicateValues" dxfId="34" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C9">
-    <cfRule type="duplicateValues" dxfId="32" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:C15">
-    <cfRule type="duplicateValues" dxfId="26" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:C17">
-    <cfRule type="duplicateValues" dxfId="24" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C21">
-    <cfRule type="duplicateValues" dxfId="18" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:C27">
-    <cfRule type="duplicateValues" dxfId="16" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C33">
-    <cfRule type="duplicateValues" dxfId="14" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35:C38">
-    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C39:C42">
-    <cfRule type="duplicateValues" dxfId="8" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C44">
-    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C50:C103">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+  <conditionalFormatting sqref="C50:C55 C57 C59:C103">
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>